<commit_message>
docs(order-management): lock 24.8 scope — payment_type/memo migration, nullable stripe cols + cron guard, mapper ownership, chargebacks display-only
</commit_message>
<xml_diff>
--- a/order_management/24.8-payment-plan-management/24.8 - Payment Plan Management.xlsx
+++ b/order_management/24.8-payment-plan-management/24.8 - Payment Plan Management.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +85,18 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,11 +118,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -150,6 +178,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -566,7 +606,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>13 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 0 out of scope.</t>
+          <t>Scope locked 2026-07-03 (Step-1 gate complete — 13 rows + 4 decisions). 13 to implement here (24.8-l = display half; automation in register). Release model: ship-together.</t>
         </is>
       </c>
     </row>
@@ -588,7 +628,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Story 24.8 asks for an admin Order Management screen to manage an order's payment plan: view scheduled/completed installments (Invoice #, Payment Type, Date, Status, Payment Memo, Amount Due, Total, Amount Paid), edit future installment dates, mark installments Paid/Unpaid/Refund, delete and add installments, enforce a post-payment lock (Refund-only), reconcile a per-order Unallocated Balance, apply the 60/30-day date rules (with authorized-user warn-not-block bypass), and drive QuickBooks actions off a per-installment milestone status. There is NO order module/controller in any repo (verified), so the entire API/UI is net-new, but the core primitives ARE built and written by the checkout/webhook/cron flows: PaymentTransaction (one row per installment with amount, due_date, status, paid_at, invoice_id), Order totals (total, paid_amount, paid_in_full_at), Invoice.invoice_number, and the reusable 60/30-day util on the cart side. Overall feasibility is mostly Deliverable. The real gaps, all confirmed against the referenced Milestone Status sheet: missing per-installment Payment Type / Payment Memo columns; NOT-NULL Stripe columns on PaymentTransaction that block non-card (Check/Wire/ACH) manual installments which the sheet explicitly requires; an absent Stripe-refund execution path (the sheet requires a real card refund); and a completely absent QuickBooks integration plus three missing Chargeback milestone statuses that themselves depend on unhandled Stripe dispute webhooks.</t>
+          <t>Payment-plan CRUD over PaymentTransactions: C13 mapper + 4 additive routes; D2 payment_type (CartPaymentMethod reuse, backfill credit_card NOT NULL) + payment_memo; D3 nullable Stripe cols + charge-cron guard; D4 admin_manual source; Mark-Paid PATCH owned here (24.15 stop-condition); Refund delegated to 24.9; chargebacks display-only (QB -&gt; epic 65, trio ND + BA flag). 12 Deliverable + 1 split.</t>
         </is>
       </c>
     </row>
@@ -613,7 +653,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -623,7 +663,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -633,7 +673,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -664,7 +704,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete)</t>
         </is>
       </c>
     </row>
@@ -790,7 +830,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -807,7 +847,7 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -822,12 +862,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Most fields are backed by built, written columns: Invoice # via PaymentTransaction.invoice_id -&gt; Invoice.invoice_number (set by webhook), Date via due_date/paid_at, Status via PaymentTransactionStatus, Amount Due via PaymentTransaction.amount, Total via Order.total, Amount Paid via Order.paid_amount (bumped by webhook). MISSING two display fields with no producing column: (1) 'Payment Type' (sheet shows Card/Check/Wire-ACH) — the only such taxonomy is the CartPaymentMethod enum on CartPaymentPlanEntry, which is NOT carried onto PaymentTransaction (PaymentTransactionSource is audit-only: checkout/cron/manual_retry/subscription_renewal); (2) 'Payment Memo' (sheet's QuickBooks Memo / Internal Comment columns, mandatory for non-CC/refund) — no memo column exists on PaymentTransaction. The list endpoint itself is net-new.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable: the two missing columns are D2's story-owned migration (payment_type reusing CartPaymentMethod, backfill credit_card NOT NULL no default; payment_memo nullable Text, service-mandatory for non-CC; doc-comments on enum declaration AND column: credit_card = Stripe card charge, sole non-manual value). Row shape = C13 mapper built here, reused by 24.7/24.6-p,q/24.15. Order.payment_memo (24.14) is order-level — deliberately distinct from per-installment memo (BA note).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2056 (PaymentTransaction: amount, due_date, status, paid_at, invoice_id), schema.prisma:1966 (Invoice.invoice_number), schema.prisma:1574 (Order.paid_amount), schema.prisma:503 (PaymentTransactionSource is audit-only), schema.prisma:2751 (CartPaymentMethod enum lives on CartPaymentPlanEntry, not PaymentTransaction); no memo/payment_type column found on PaymentTransaction</t>
+          <t>admin schema PT :2073-2110, invoice_id :2093, Invoice.invoice_number :1981, Order.total :1552, paid_amount :1578 (gross per 24.9 D3), Order.payment_memo :1576; deriveBalanceDue orders.helpers.ts:33</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -848,7 +888,7 @@
       </c>
       <c r="L2" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: upgraded Partial -&gt; Deliverable; D2 recorded.</t>
         </is>
       </c>
     </row>
@@ -880,12 +920,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>PaymentTransaction.due_date is a real, written column that the charge cron reads (WHERE status='scheduled' AND due_date&lt;=now). A net-new admin PATCH endpoint can update due_date for scheduled installments. No new primitive needed.</t>
+          <t>CONFIRMED 2026-07-03. due_date NOT NULL + [status,due_date] index; charge cron picks scheduled+due, so a date edit composes cleanly. AGREED GUARD: scheduled-only. Date validation via 24.8-j/k.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2069 (due_date), schema.prisma:2082 (@@index([status, due_date])); background-worker-service/src/jobs/payment-charge/payment-charge.service.ts:62-67 (findMany WHERE status=scheduled AND due_date&lt;=now)</t>
+          <t>admin schema due_date :2086, index :2103; worker payment-charge.service.ts:62-67</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -902,7 +942,7 @@
       </c>
       <c r="L3" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; scheduled-only guard.</t>
         </is>
       </c>
     </row>
@@ -934,12 +974,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>PaymentTransactionStatus enum includes succeeded(=Paid)/scheduled(=Unpaid). A net-new admin endpoint can write the status (plus paid_at). The sheet confirms manual mark-as-Paid is required for Check/Wire/ACH; the status write itself is deliverable on existing fields (the mandatory-memo capture for manual payments rides on the missing memo column tracked under 24.8-a). Caveat to flag: the webhook is the real source of card paid status, so a manual override is a status flag only, not a real charge.</t>
+          <t>CONFIRMED 2026-07-03. Mark-as-Paid/Unpaid PATCH OWNED HERE (reassigned from 24.7; 24.7 consumes). Paid =&gt; succeeded + paid_at; Unpaid =&gt; scheduled + cleared. AGREED: manual-method installments only — service rejects hand-marking credit_card rows (webhook stays card source of truth; this IS 24.7-b's gate, built here). Mark-Paid bumps paid_amount/paid_in_full_at mirroring webhook; Unpaid reverses (the one legitimate gross decrement — bookkeeping correction, not refund). This PATCH is 24.15's stop-condition.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:491-500 (enum PaymentTransactionStatus: scheduled/processing/succeeded/failed/canceled/refunded); external-api-service/src/modules/webhook/services/webhook.service.ts:2089-2103 (webhook owns status + paid_amount writes today)</t>
+          <t>admin schema enum :491-500; ext webhook.service.ts:2111-2125 (write pattern)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -956,7 +996,7 @@
       </c>
       <c r="L4" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; manual-only gate + bookkeeping semantics.</t>
         </is>
       </c>
     </row>
@@ -973,7 +1013,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -988,17 +1028,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Setting PaymentTransaction.status=refunded and voiding the linked invoice is implemented logic (handleChargeRefunded), so the status flip is deliverable. BUT the milestone sheet's Refunded status explicitly requires refunding the payment back to the credit card (money movement), and there is NO admin-initiated refund execution: grep for refunds.create / stripe.refunds across all repos returns NOTHING. Today refunds only happen when performed OUTSIDE the system and Stripe fires charge.refunded. A true money-back Refund from this screen is not built.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable (sequenced on 24.9). The Refund action IS 24.9's per-installment primitive (POST /orders/:id/refunds with payment_transaction_id: cap, mandatory reason, Manual/Stripe branch, ledger row, refunded/refund_failed flip). 24.8 OWNS NO REFUND CODE — plan view only exposes the action. Dependency owner corrected from generic 'Payments/Checkout' to 24.9.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>external-api-service/src/modules/webhook/services/webhook.service.ts:2879 (handleChargeRefunded flips status + voids invoice); external-api-service/src/modules/webhook/controllers/webhook.controller.ts:186 (only reacts to charge.refunded fired externally); grep refunds.create|stripe.refunds across all repos = none found (the only .refund() hits are PPL lead-credit refunds, not Stripe)</t>
+          <t>ext webhook.service.ts:3038 (amount-aware change owned by 24.9 D2); grep refunds.create = zero pre-24.9; 24.9 doc D1</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Stripe refund execution (stripe.refunds.create) is unbuilt — gates the money-movement half of this action</t>
+          <t>24.9 (SBE-1133) refunds endpoint + ledger — same release, builds first</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -1014,7 +1054,7 @@
       </c>
       <c r="L5" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: upgraded Partial -&gt; Deliverable (delegated to 24.9).</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1086,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>PaymentTransaction rows are deletable; a net-new admin DELETE endpoint can remove a scheduled (unpaid) installment. The model exists and is the per-installment unit.</t>
+          <t>CONFIRMED 2026-07-03. PT is the per-installment unit; DELETE unblocked. AGREED GUARD: scheduled-only (succeeded = lock; processing = mid-charge; canceled/refunded = audit trail). Allocation return free — balance derived, deletion IS the return. Audit in-tx with snapshot.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2056 (PaymentTransaction model, one row per installment)</t>
+          <t>admin schema PT :2073-2110</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1068,7 +1108,7 @@
       </c>
       <c r="L6" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; scheduled-only guard.</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1125,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1100,12 +1140,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>A net-new admin POST can create a PaymentTransaction, but the model mandates NOT-NULL stripe_payment_method_id, stripe_customer_id and idempotency_key (designed for the off-session card cron). The milestone sheet explicitly requires non-card payment types (Check, Wire/ACH) with manual mark-as-Paid, and such installments cannot satisfy those NOT-NULL Stripe columns without schema relaxation. Card-based manual installments are addable when the customer has a saved PM; non-card manual installments need schema work.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable: gaps became D2/D3/D4 story-owned migration work. POST creates scheduled PT: amount, due_date, payment_type (D2), payment_memo (mandatory non-CC), null Stripe ids for manual types (D3 — doc-comments: null = manual installment, no Stripe identity), app-UUID idempotency_key, source admin_manual (D4). Guards: unallocated cap (i), 60/30 two-phase (j/k), audit. CARD-SIBLING CONSTRAINT: manual credit_card installment requires existing Stripe identity on the order (ids copied from sibling card rows) else rejected. COMPANIONS: 5 writer updates (all verified card flows at gate) + worker charge/retry cron guard payment_type=credit_card.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2067 (stripe_payment_method_id NOT NULL), :2068 (stripe_customer_id NOT NULL), :2076 (idempotency_key NOT NULL unique); created today only by exhibitor-backend-api/src/payments/services/payments.service.ts:261 and external-api-service/src/modules/webhook/services/webhook.service.ts:730</t>
+          <t>admin schema :2084/:2085 (D3 nullable), :2094 (stays NOT NULL); creation sites verified: exh payments :261, cart :1370, ppl checkout :227; ext webhook :730; admin :969</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1122,7 +1162,7 @@
       </c>
       <c r="L7" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: upgraded Partial -&gt; Deliverable; D2/D3/D4 recorded.</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1194,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Paid state is determinable from built, written fields: PaymentTransaction.status=succeeded/paid_at and Order.paid_in_full_at (set by webhook). New service logic can gate edit/delete/add against these and allow only the refund path. No new primitive needed.</t>
+          <t>CONFIRMED 2026-07-03. PLAN-LEVEL LOCK = Order.paid_in_full_at set; before that, settled installments individually immutable while scheduled rows stay editable (restructuring intent). Lock = invariant the per-row guards jointly enforce; residual = explicit consistent locked-error shape + tests. Refund stays available via 24.9.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1575 (Order.paid_in_full_at), schema.prisma:2071 (PaymentTransaction.paid_at); external-api-service/src/modules/webhook/services/webhook.service.ts:2089-2103 (webhook sets paid_amount + paid_in_full_at)</t>
+          <t>admin schema paid_in_full_at :1579, PT.paid_at :2088; ext webhook.service.ts:2111-2125</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1176,7 +1216,7 @@
       </c>
       <c r="L8" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; plan-level lock semantics.</t>
         </is>
       </c>
     </row>
@@ -1208,12 +1248,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>There is no stored 'Unallocated Balance' field, but it is fully derivable as Order.total minus the sum of allocated installment amounts (PaymentTransaction.amount). New service logic computes it on each mutation. All inputs are built/written columns; restructuring is just composition of add/edit/delete on PaymentTransaction.</t>
+          <t>CONFIRMED 2026-07-03. DERIVED, NEVER STORED (no unallocated column anywhere): Order.total − Σ PT.amount, Decimal floored-0 fixed-2. 'Move back' automatic — deletion shrinks the Σ. Surfaced in GET payment-plan.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1551 (Order.total), schema.prisma:2062 (PaymentTransaction.amount); no 'unallocated' column exists</t>
+          <t>admin schema Order.total :1552, PT.amount :2079; deriveBalanceDue orders.helpers.ts:33</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1234,7 +1274,7 @@
       </c>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; derived-not-stored.</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1306,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Same derivation as 24.8-h (total - sum(installment amounts) &gt; 0). Net-new validation logic on built fields; nothing upstream missing.</t>
+          <t>CONFIRMED 2026-07-03. Guard on the POST: reject when unallocated &lt;= 0; cap amount &lt;= unallocated; computed INSIDE the same transaction as the insert (no stale-balance race). 'Unless deleted/adjusted' needs no code.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1551 (Order.total), schema.prisma:2062 (PaymentTransaction.amount)</t>
+          <t>same as 24.8-h</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1288,7 +1328,7 @@
       </c>
       <c r="L10" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; in-tx guard.</t>
         </is>
       </c>
     </row>
@@ -1320,12 +1360,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>The exact 60/30-day rule logic already exists and is reusable: computePaymentDateWarnings + assertNoPaymentDateAfterShow in the cart util. The 'first show date' is derivable on the order side via OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows.date (no-op for non-show/undated orders, mirroring the cart util which filters null dates). Wiring the util to order data is net-new but trivial on built primitives.</t>
+          <t>CONFIRMED 2026-07-03. Shipped util current: 60/30 windows :9-10, assertPaymentPlanTotal :18, assertNoPaymentDateAfterShow :40, computePaymentDateWarnings :56. Net-new = composition: first show date via OrderItem.show_product_id :1955 -&gt; ShowProduct :2659 -&gt; Shows :2388. AGREED: null show date =&gt; skip window checks + 'no show date on file' warning. Plan-time: share the util (import/hoist), don't duplicate.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/cart/utils/cart-payment-plan.util.ts:36-49 (assertNoPaymentDateAfterShow) + :54-79 (computePaymentDateWarnings 60/30 logic); admin-backend-api/prisma/schema.prisma:1940 (OrderItem.show_product_id) -&gt; :2640 (ShowProduct) -&gt; Shows.date (nullable)</t>
+          <t>admin cart-payment-plan.util.ts (refs above); schema :1955/:2659/:2388 (Shows.date nullable)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1342,7 +1382,7 @@
       </c>
       <c r="L11" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; null-show-date handling agreed.</t>
         </is>
       </c>
     </row>
@@ -1374,12 +1414,12 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Role/permission infra exists (cart.manage-payment-plan permission, role seeder) and the warning-not-block pattern is already implemented on the cart side: computePaymentDateWarnings returns a non-blocking warnings[] array surfaced to the FE, and upsertPlan threads a confirm flag. Re-applying the same pattern to the order endpoint behind the role gate is net-new but fully backed.</t>
+          <t>CONFIRMED 2026-07-03. Port the live two-phase pattern: no confirm =&gt; {plan, warnings[]}; ?confirm=true =&gt; execute (cart-payment-plan.service.ts:54-108; cart.controller.ts:1246-1283). 'Authorized users' = the route's own orders.payment-plan.* permission key (mirrors cart.manage-payment-plan, cart.constants.ts:54, role.seeder.ts:238) — no second bypass permission.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/cart/services/cart-payment-plan.service.ts:54-108 (upsertPlan returns warnings + confirm flag); admin-backend-api/src/admin/cart/constants/cart.constants.ts:43 (MANAGE_PAYMENT_PLAN='cart.manage-payment-plan'); admin-backend-api/src/database/seeds/role.seeder.ts:219</t>
+          <t>as cited</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1396,7 +1436,7 @@
       </c>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable; two-phase port.</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1453,7 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Split: Deliverable (display) / automation in register</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1428,17 +1468,17 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>The referenced sheet was read: it defines 8 milestone statuses (Paid, Unpaid, Chargeback Pending, Chargeback Lost, Chargeback Won, CC Failed, Voided, Refunded). TWO gaps. (1) Taxonomy: 5 map to the existing enum (succeeded/scheduled/failed/canceled/refunded) but the 3 Chargeback statuses are entirely absent AND depend on Stripe charge.dispute.* webhooks that the webhook switch does not handle. (2) QuickBooks: NO integration code anywhere (only dormant quickbooks_* columns + QuickBooksSyncStatus enum; product-management DTOs explicitly say 'until QuickBooks integration ships'). The required per-status QuickBooks actions (Received Payment, credit memo, journal entries) cannot be executed until a QuickBooks integration is built.</t>
+          <t>DECIDED 2026-07-03 (D1): DISPLAY-ONLY. Display half ships — C13 mapper carries milestone status mapped from statuses this release produces (6 enum values + 24.9's refund_failed). Automation split by cause: QuickBooks actions = Out of Scope citing epic 65 'Quickbooks Integration/Invoice Creation Process' (Admin Panel Page 2, 65.1-65.5, NOT in Jira; consistent with 24.9-i/24.6); chargeback trio (Pending/Won/Lost) = Not Deliverable — no charge.dispute.* handling, no enum values, NO OWNING STORY anywhere; BA FLAG: the Milestone Status sheet references statuses no story produces. Exhibitor SETTLED/NON_PAYABLE watch stays scoped to refund_failed (actioned in 24.9).</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1567 (Order.quickbooks_* columns) + :474 (QuickBooksSyncStatus enum, no producer); admin-backend-api/src/admin/product-management/product-management.service.ts:162 ('QuickBooks integration (future module)'); grep intuit|node-quickbooks|qbo across all repos = none; schema.prisma:491-500 (enum lacks the 3 chargeback statuses); external-api-service/src/modules/webhook/controllers/webhook.controller.ts:153-191 (no charge.dispute.* case)</t>
+          <t>admin schema quickbooks_* :1569-1571 dormant, QuickBooksSyncStatus :474 writer-less; grep intuit/qbo = none; ext webhook.controller.ts:154-188 (no dispute cases); enum :491-500; Jira 'QuickBooks' = zero issues</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks integration (Intuit/QBO client + per-status actions) AND Stripe dispute/chargeback webhook handling AND the 3 missing chargeback milestone statuses are all unbuilt</t>
+          <t>QB actions: epic 65, Admin Panel Page 2 (un-ticketed). Chargebacks: no owning story — BA flag.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1454,7 +1494,7 @@
       </c>
       <c r="L13" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — QuickBooks integration (Intuit/QBO client + per-status actions) AND Stripe dispute/chargeback webhook handling AND the 3 missing chargeback milestone statuses are all unbuilt)</t>
+          <t>Gate 2026-07-03: split verdict (D1 display-only).</t>
         </is>
       </c>
     </row>
@@ -1486,12 +1526,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>All enforcement inputs are built: Order.total / paid_amount, PaymentTransaction.amount/status/due_date, the reusable 60/30 util, and the derivable allocation. Implementing enforcement in the net-new order payment-plan service is straightforward composition of the above (mirrors assertPaymentPlanTotal on the cart side).</t>
+          <t>CONFIRMED 2026-07-03. Composite of confirmed guards: totals (assertPaymentPlanTotal), allocation (in-tx derived), date rules (two-phase port), eligibility gates (b/c/e/f), plan lock (g) — all service/tx-side. C8/C9 residuals: seed orders.payment-plan.* keys + one audit record per mutating tx.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/cart/utils/cart-payment-plan.util.ts:18-33 (assertPaymentPlanTotal); schema.prisma:1551 (Order.total), :1574 (paid_amount), :2062 (PaymentTransaction.amount)</t>
+          <t>cart-payment-plan.util.ts:18; schema :1552/:1578/:2079; admin-audit.service.ts:50</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1512,7 +1552,7 @@
       </c>
       <c r="L14" s="13" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1593,15 +1633,19 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Return the order's installments with Invoice #, date, status, amount due, order total, amount paid, plus computed Unallocated Balance and 60/30-day warnings.</t>
+          <t>Installment rows via the C13 mapper (8 columns + milestone status) + derived Unallocated Balance + 60/30 warnings.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>24.8-a, 24.8-h, 24.8-i</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>24.8-a, h, i, l(display)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mapper reused by 24.7 GET payments, 24.6-p/q, 24.15 cron</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1616,7 +1660,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Manually add a new installment; validates Unallocated Balance remains, runs the 60/30-day rule (warn/bypass), enforces totals server-side.</t>
+          <t>Add installment: D2/D3/D4 fields, unallocated + 60/30 two-phase (?confirm=), card-sibling constraint, audit in-tx.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1639,15 +1683,19 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Edit a future installment's date or mark it Paid/Unpaid/Refund; enforces post-payment lock, date rules with warning-bypass, milestone status, backend total enforcement.</t>
+          <t>Edit future date (scheduled-only) or Mark Paid/Unpaid (manual-method-only; paid_amount bookkeeping mirror/reverse); post-payment lock; two-phase warnings; audit in-tx. Refund NOT here — delegated to 24.9's refunds endpoint.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>24.8-b, 24.8-c, 24.8-d, 24.8-g, 24.8-j, 24.8-k, 24.8-l, 24.8-m</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>24.8-b, c, g, j, k, m</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Mark-Paid = 24.15's stop-condition; consumed by 24.7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1662,7 +1710,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Delete an unpaid installment and return its amount to the Unallocated Balance; blocked when already paid.</t>
+          <t>Delete a scheduled installment (derived balance auto-returns); post-payment lock; audit in-tx with snapshot.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1671,6 +1719,60 @@
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Migration (admin, mirrors x4)</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>payment_type (CartPaymentMethod, backfill credit_card, NOT NULL, no default) + payment_memo (nullable Text) + nullable stripe_payment_method_id/stripe_customer_id + admin_manual source + doc-comments (enum declaration, payment_type, both nullable cols).</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>24.8-a, f (D2/D3/D4)</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>24.7 classification, 24.9-f unblock, 24.15 selection</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Writer updates (5 sites) + cron guard</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Set payment_type: credit_card explicitly at exh payments :261, cart :1370, ppl checkout :227; ext webhook :730; admin :969. Worker charge+retry queries add payment_type=credit_card guard.</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>24.8-f companions</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>exhibitor/external/worker repos — in-release</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1683,54 +1785,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="D1" s="16" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>The Milestone Status sheet lists Chargeback Pending / Chargeback Won / Chargeback Lost as payment-plan milestone statuses, but they require Stripe charge.dispute.* webhook handling (not implemented) and QuickBooks journal entries. Is automating these chargeback statuses in scope for THIS Payment Plan Management story, or owned by a separate Payments/dispute-handling epic that this screen merely displays?</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>OPEN — for team discussion</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): (pending). Current leaning is that chargeback-status automation (Stripe dispute webhooks + QuickBooks journal entries) belongs to a separate Payments/dispute-handling epic and this screen merely DISPLAYS those statuses; 24.8-l stays Blocked until the team confirms scope. No code until answered.</t>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>24.8-l</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>QuickBooks per-status actions</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Out of Scope</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>QB integration to execute the sheet's per-status actions (Received Payment, credit memo, journal entries)</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Epic 65, Admin Panel Page 2 (un-ticketed; no Jira issues)</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>— (BA)</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>Not commissioned</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Display half ships in 24.8; captured statuses + ledger are what the future sync consumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>24.8-l</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Chargeback trio (Pending/Won/Lost)</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Not Deliverable</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>charge.dispute.* webhook handling + 3 enum values + an owning story — none exist anywhere</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>none — no owning story</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>— (BA)</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>BA FLAG: Milestone Status sheet references statuses no story produces (same pattern as epic 65 missing refund story).</t>
         </is>
       </c>
     </row>
@@ -1771,53 +1961,53 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Stripe refund execution (stripe.refunds.create) — no refund-issuing code exists in any repo; the charge.refunded webhook only reacts to refunds performed externally. The Milestone sheet's Refunded status requires a real refund to the card.</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>24.8-d (Mark as Refund money-movement)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Payments / Checkout integration (external-api-service Stripe module)</t>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Refund execution (per-installment primitive + ledger + wrapper)</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>24.8-d</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>24.9 (SBE-1133) — same release, builds first</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>QuickBooks integration (Intuit/QBO API client) plus per-installment milestone-status actions per the approved process document — only dormant quickbooks_* columns and a sync-status enum exist; nothing writes QuickBooks.</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>24.8-l (milestone status -&gt; QuickBooks actions)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>QuickBooks / Billing integration epic</t>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>QuickBooks integration</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>24.8-l automation half</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Epic 65 'Quickbooks Integration/Invoice Creation Process', Admin Panel Page 2 (un-ticketed; lacks dispute story too — BA flagged)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Stripe dispute/chargeback webhook handling (charge.dispute.created/updated/closed) plus the 3 missing Chargeback milestone statuses on PaymentTransactionStatus — the webhook switch handles no dispute events and the enum lacks these statuses.</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>24.8-l (Chargeback Pending/Won/Lost milestone statuses)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Payments / dispute-handling integration</t>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Downstream consumers (NOT dependencies): 24.7 (mapper + Mark-Paid gate + classification), 24.6-p/q (mapper), 24.15 (stop-condition + scan + cron guard), 24.9-f manual half (unblocked by D2/D3), 13.3-t/SBE-1154 (taxonomy aligned)</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1832,7 +2022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1852,110 +2042,158 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>Not started — analysis/feasibility stage only. No branch, no SBE ticket, no PR, no Swagger tag. Entire API is net-new (no order module/controller in any repo). Per-requirement build status is ◻ Not started.</t>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03; scope + 4 decisions locked (D1 display-only chargebacks; D2 payment_type/payment_memo w/ comments; D3 nullable Stripe cols + cron guard; D4 admin_manual). Release model: all remaining OM stories ship together; refund action delegated to 24.9.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>Branch / PR</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Remaining — all in-scope</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Everything is remaining (nothing built): 24.8-a, 24.8-b, 24.8-c, 24.8-d, 24.8-e, 24.8-f, 24.8-g, 24.8-h, 24.8-i, 24.8-j, 24.8-k, 24.8-l, 24.8-m.</t>
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>SBE-1132 (In Progress, Prantik Saha)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>Open decision — chargeback milestone scope</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Are Chargeback Pending/Won/Lost statuses (Stripe charge.dispute.* webhooks + QuickBooks journal entries) in scope for this story or a separate Payments/dispute epic this screen merely displays? Gates 24.8-l. No code until answered.</t>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Deferred — 24.8-l</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Milestone status → QuickBooks actions BLOCKED: needs QuickBooks (Intuit/QBO) integration + per-status actions, Stripe dispute/chargeback webhook handling, and the 3 missing Chargeback statuses on PaymentTransactionStatus. None exist today.</t>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Dependency — Payments/Checkout</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Stripe refund execution (stripe.refunds.create) — needed for 24.8-d money-movement refund; no refund-issuing code exists in any repo.</t>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Dependency — QuickBooks/Billing</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>QuickBooks integration (Intuit/QBO API client) + per-installment milestone-status actions — needed for 24.8-l.</t>
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Dependency — Payments/dispute-handling</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Stripe dispute/chargeback webhook handling (charge.dispute.created/updated/closed) + the 3 missing Chargeback milestone statuses — needed for 24.8-l.</t>
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>24.8-a…m (l = display half) — one migration (D2+D3+D4) + 4 routes + C13 mapper + cron guard + 5 writer updates + permission seeds + audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>All confirmed scope unbuilt</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Not ready — see Open Questions</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>24.8-l automation half (QB -&gt; epic 65; chargeback trio -&gt; no owning story, BA flag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>24.9 refund stack (same release); QuickBooks epic 65 (un-ticketed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Front-end wiring.</t>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Payment Plan screen FE wiring</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.8 Payment Plan Management — correct D2 card-writer count 5 -> 7
Exhaustive PT-creation sweep across all 5 repos (2026-07-06) confirms 8
paymentTransaction create/upsert sites: 7 pre-existing card writers (exhibitor
x4 — cart:1474, payments:267, ppl/checkout:253, ppl/ppl.service:2537; external
x2 — webhook:752 create + :1152 upsert; admin x1 — ppl-service-provider:970),
all tagging payment_type: credit_card explicitly, plus 24.8's own manual-add
writer (order-payment-plan:270, source admin_manual). The gate's D2 estimate of
5 undercounted by two (exhibitor ppl.service + external webhook upsert). Not a
delivery gap — payment_type is NOT NULL no default and gates are green, so every
active card writer is tagged. Corrected D2, Confirmed build scope, 24.8-f
evidence, Endpoints writer row, consolidation note in .md + .xlsx.
</commit_message>
<xml_diff>
--- a/order_management/24.8-payment-plan-management/24.8 - Payment Plan Management.xlsx
+++ b/order_management/24.8-payment-plan-management/24.8 - Payment Plan Management.xlsx
@@ -1146,12 +1146,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable: gaps became D2/D3/D4 story-owned migration work. POST creates scheduled PT: amount, due_date, payment_type (D2), payment_memo (mandatory non-CC), null Stripe ids for manual types (D3 — doc-comments: null = manual installment, no Stripe identity), app-UUID idempotency_key, source admin_manual (D4). Guards: unallocated cap (i), 60/30 two-phase (j/k), audit. CARD-SIBLING CONSTRAINT: manual credit_card installment requires existing Stripe identity on the order (ids copied from sibling card rows) else rejected. COMPANIONS: 5 writer updates (all verified card flows at gate) + worker charge/retry cron guard payment_type=credit_card.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable: gaps became D2/D3/D4 story-owned migration work. POST creates scheduled PT: amount, due_date, payment_type (D2), payment_memo (mandatory non-CC), null Stripe ids for manual types (D3 — doc-comments: null = manual installment, no Stripe identity), app-UUID idempotency_key, source admin_manual (D4). Guards: unallocated cap (i), 60/30 two-phase (j/k), audit. CARD-SIBLING CONSTRAINT: manual credit_card installment requires existing Stripe identity on the order (ids copied from sibling card rows) else rejected. COMPANIONS: 7 card-writer updates (exhibitor x4, external x2, admin x1; corrected 2026-07-06 from gate estimate of 5, exhaustive PT-creation sweep) + worker charge/retry cron guard payment_type=credit_card.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin schema :2084/:2085 (D3 nullable), :2094 (stays NOT NULL); creation sites verified: exh payments :261, cart :1370, ppl checkout :227; ext webhook :730; admin :969</t>
+          <t>admin schema :2084/:2085 (D3 nullable), :2094 (stays NOT NULL); creation sites verified via exhaustive sweep 2026-07-06 -- 7 pre-existing card writers, not the gate's 5: exhibitor cart:1474, payments:267, ppl/checkout:253, ppl/ppl.service:2537; external webhook:752 (create) + :1152 (upsert); admin ppl-service-provider-detail-view:970 -- all now set credit_card explicitly. The 8th PT writer, admin order-payment-plan:270, is 24.8's own manual-add (payment_type from DTO, source admin_manual).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Writer updates (5 sites) + cron guard</t>
+          <t>Writer updates (7 card sites) + cron guard</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Set payment_type: credit_card explicitly at exh payments :261, cart :1370, ppl checkout :227; ext webhook :730; admin :969. Worker charge+retry queries add payment_type=credit_card guard.</t>
+          <t>Set payment_type: credit_card explicitly at the 7 pre-existing card PT-creation sites -- exhibitor cart.service.ts:1474, payments.service.ts:267, ppl/checkout.service.ts:253, ppl/ppl.service.ts:2537; external webhook.service.ts:752 (create) + :1152 (upsert); admin ppl-service-provider-detail-view.service.ts:970. (8th PT writer admin order-payment-plan.service.ts:270 is 24.8's own manual-add: payment_type from DTO, source admin_manual.) Worker charge+retry queries add payment_type=credit_card guard. [Count corrected 2026-07-06 from gate's 5.]</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">

</xml_diff>